<commit_message>
Refine HORIZONS call sheets, compact cards, brand styling, and trackers
</commit_message>
<xml_diff>
--- a/HORIZONS_Website_Update_Tracker.xlsx
+++ b/HORIZONS_Website_Update_Tracker.xlsx
@@ -23,19 +23,20 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Completed Website Updates" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Website Change Requests'!$A$1:$K$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'START HERE'!$A$1:$A$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Website Change Requests'!$A$1:$K$204</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Missing Information'!$A$1:$J$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Questions To Answer'!$A$1:$K$201</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Schedule Updates'!$A$1:$O$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Schedule Updates'!$A$1:$O$202</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Task Updates'!$A$1:$M$201</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Contact Updates'!$A$1:$O$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Contact Updates'!$A$1:$O$203</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Supplier Updates'!$A$1:$R$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Podcast Updates'!$A$1:$M$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Content Capture Updates'!$A$1:$N$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Documents + Links'!$A$1:$K$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Red Flags + Decisions'!$A$1:$M$201</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Image + Asset Updates'!$A$1:$I$201</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Completed Website Updates'!$A$1:$H$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Image + Asset Updates'!$A$1:$I$203</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Completed Website Updates'!$A$1:$H$202</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -69,7 +70,7 @@
       <color rgb="006A4B13"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -86,8 +87,18 @@
         <fgColor rgb="00FBF8F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7F0E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFECE6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -109,11 +120,16 @@
         <color rgb="00DED1BF"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00DED1BF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -130,6 +146,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,7 +529,7 @@
   <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="112" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,6 +539,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -515,6 +547,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -523,125 +556,132 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Set Status clearly. Only Approved or Ready for Codex rows should normally be applied to the live website.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Use Needs Confirmation when spelling, timing, ownership, files, or approvals are uncertain.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Codex uses this tracker to update the official website source data in content.json after review.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Website comments are discussion and feedback. They do not automatically change official website data.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Chris name rule: there is only one Chris, and his name is Chris Manoe.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>HORIZONS Hall rule: do not use Farmers Market Stage.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Do not invent missing phone numbers, emails, files, timings, or approvals.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Excel cannot use / in tab names, so Image / Asset Updates is named Image + Asset Updates.</t>
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="9" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n"/>
+    </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Allowed status values</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Needs Confirmation</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Ready for Codex</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>Added to Website</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Rejected / Do Not Add</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Waiting on Info</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:A24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -655,89 +695,89 @@
   <dimension ref="A1:N201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Content Update ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Day / Date</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Moment / Capture Item</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Content Type</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Person Responsible</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>Approved By</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="N1" s="8" t="inlineStr">
         <is>
           <t>Website Update Status</t>
         </is>
@@ -3945,7 +3985,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:N201"/>
-  <dataValidations count="3">
+  <dataValidations count="6">
     <dataValidation sqref="K2:K201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
@@ -3954,6 +3994,15 @@
     </dataValidation>
     <dataValidation sqref="J2:J201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Low,Normal,High,Critical"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Critical,High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3969,71 +4018,71 @@
   <dimension ref="A1:K201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Document ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Document Title</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Day / Date</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>File Name</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>File Link / URL</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Website Location</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -6641,12 +6690,15 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K201"/>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="I2:I201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Menus,Maps,Site Map,Seating Plans,Room Layouts,Brand Files,Supplier Documents,Runbooks,Production Documents,Guest Experience,HORIZONS House,Room Drops,Swag"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6662,83 +6714,83 @@
   <dimension ref="A1:M201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="27" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Item ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Issue / Decision Needed</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Why It Matters</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Deadline</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Current Status</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Final Decision / Update</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>Approved By</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>Date Resolved</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Website Update Status</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -9746,7 +9798,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:M201"/>
-  <dataValidations count="3">
+  <dataValidations count="5">
     <dataValidation sqref="L2:L201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
@@ -9755,6 +9807,12 @@
     </dataValidation>
     <dataValidation sqref="B2:B201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Red Flag,Decision Needed,Risk,Confirmation Needed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9767,62 +9825,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I201"/>
+  <dimension ref="A1:I203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Asset ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Image / Asset Name</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>File Name</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>File Link / Location</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Description / Caption</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Alt Text</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -12028,11 +12086,108 @@
       <c r="H201" s="6" t="n"/>
       <c r="I201" s="6" t="n"/>
     </row>
+    <row r="202">
+      <c r="A202" s="9" t="inlineStr">
+        <is>
+          <t>ASSET-R2-001</t>
+        </is>
+      </c>
+      <c r="B202" s="9" t="inlineStr">
+        <is>
+          <t>Brand / Hero</t>
+        </is>
+      </c>
+      <c r="C202" s="9" t="inlineStr">
+        <is>
+          <t>Official main HORIZONS logo</t>
+        </is>
+      </c>
+      <c r="D202" s="9" t="inlineStr">
+        <is>
+          <t>horizons-main-logo-black.png</t>
+        </is>
+      </c>
+      <c r="E202" s="9" t="inlineStr">
+        <is>
+          <t>assets/logos/horizons-main-logo-black.png</t>
+        </is>
+      </c>
+      <c r="F202" s="9" t="inlineStr">
+        <is>
+          <t>Primary hero/header logo source.</t>
+        </is>
+      </c>
+      <c r="G202" s="9" t="inlineStr">
+        <is>
+          <t>Official HORIZONS logo</t>
+        </is>
+      </c>
+      <c r="H202" s="9" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="I202" s="9" t="inlineStr">
+        <is>
+          <t>Provided by Chris Manoe; do not modify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="inlineStr">
+        <is>
+          <t>ASSET-R2-002</t>
+        </is>
+      </c>
+      <c r="B203" s="9" t="inlineStr">
+        <is>
+          <t>Swag / Room Drops / HORIZONS House</t>
+        </is>
+      </c>
+      <c r="C203" s="9" t="inlineStr">
+        <is>
+          <t>Swag reference image set</t>
+        </is>
+      </c>
+      <c r="D203" s="9" t="inlineStr">
+        <is>
+          <t>assets/images/swag/*.jpeg</t>
+        </is>
+      </c>
+      <c r="E203" s="9" t="inlineStr">
+        <is>
+          <t>assets/images/swag/</t>
+        </is>
+      </c>
+      <c r="F203" s="9" t="inlineStr">
+        <is>
+          <t>Tote bag, notebook, bottle, charger, fragrances, eye mask, fan, caps, massager, pen, lanyard.</t>
+        </is>
+      </c>
+      <c r="G203" s="9" t="inlineStr">
+        <is>
+          <t>Approved swag reference images</t>
+        </is>
+      </c>
+      <c r="H203" s="9" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="I203" s="9" t="inlineStr">
+        <is>
+          <t>Added to content.json visual sections.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I201"/>
-  <dataValidations count="1">
+  <autoFilter ref="A1:I203"/>
+  <dataValidations count="2">
     <dataValidation sqref="H2:H201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12045,56 +12200,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Update ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Source Tab</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Summary of Update</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Date Completed</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Completed By</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Website Section Updated</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Commit Message</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -14100,8 +14255,50 @@
       <c r="G201" s="6" t="n"/>
       <c r="H201" s="6" t="n"/>
     </row>
+    <row r="202">
+      <c r="A202" s="9" t="inlineStr">
+        <is>
+          <t>R2-001</t>
+        </is>
+      </c>
+      <c r="B202" s="9" t="inlineStr">
+        <is>
+          <t>Website Change Requests</t>
+        </is>
+      </c>
+      <c r="C202" s="9" t="inlineStr">
+        <is>
+          <t>Round two navigation, Call Sheet, compact card, official logo, and swag image update</t>
+        </is>
+      </c>
+      <c r="D202" s="9" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="E202" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F202" s="9" t="inlineStr">
+        <is>
+          <t>Overview / Schedule / Call Sheet / Flights / Suppliers / Content / Swag</t>
+        </is>
+      </c>
+      <c r="G202" s="9" t="inlineStr">
+        <is>
+          <t>Refine HORIZONS call sheets, compact cards, brand styling, and trackers</t>
+        </is>
+      </c>
+      <c r="H202" s="9" t="inlineStr">
+        <is>
+          <t>Pending deployment confirmation.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H201"/>
+  <autoFilter ref="A1:H202"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14112,74 +14309,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K201"/>
+  <dimension ref="A1:K204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Request ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Date Added</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Added By</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Current Website Text / Issue</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>Requested Change</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Reason / Context</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>Approved By</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -16785,14 +16982,191 @@
       <c r="J201" s="6" t="n"/>
       <c r="K201" s="6" t="n"/>
     </row>
+    <row r="202">
+      <c r="A202" s="9" t="inlineStr">
+        <is>
+          <t>WCR-R2-001</t>
+        </is>
+      </c>
+      <c r="B202" s="9" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C202" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D202" s="9" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="E202" s="9" t="inlineStr">
+        <is>
+          <t>Side progress index could stick around Red Flags.</t>
+        </is>
+      </c>
+      <c r="F202" s="9" t="inlineStr">
+        <is>
+          <t>Replace scroll spy with sticky-header aware active section tracking.</t>
+        </is>
+      </c>
+      <c r="G202" s="9" t="inlineStr">
+        <is>
+          <t>CEO round-two review</t>
+        </is>
+      </c>
+      <c r="H202" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I202" s="9" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J202" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K202" s="9" t="inlineStr">
+        <is>
+          <t>Implemented in script.js.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="inlineStr">
+        <is>
+          <t>WCR-R2-002</t>
+        </is>
+      </c>
+      <c r="B203" s="9" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C203" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D203" s="9" t="inlineStr">
+        <is>
+          <t>Call Sheet</t>
+        </is>
+      </c>
+      <c r="E203" s="9" t="inlineStr">
+        <is>
+          <t>No dedicated Daily Call Sheet view.</t>
+        </is>
+      </c>
+      <c r="F203" s="9" t="inlineStr">
+        <is>
+          <t>Add Daily Call Sheet section rendered from schedule data.</t>
+        </is>
+      </c>
+      <c r="G203" s="9" t="inlineStr">
+        <is>
+          <t>CEO round-two review</t>
+        </is>
+      </c>
+      <c r="H203" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I203" s="9" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J203" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K203" s="9" t="inlineStr">
+        <is>
+          <t>Implemented in index.html/script.js.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="9" t="inlineStr">
+        <is>
+          <t>WCR-R2-003</t>
+        </is>
+      </c>
+      <c r="B204" s="9" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C204" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D204" s="9" t="inlineStr">
+        <is>
+          <t>Cards</t>
+        </is>
+      </c>
+      <c r="E204" s="9" t="inlineStr">
+        <is>
+          <t>Travel, supplier, and content capture cards were too long.</t>
+        </is>
+      </c>
+      <c r="F204" s="9" t="inlineStr">
+        <is>
+          <t>Use compact default cards with expandable details.</t>
+        </is>
+      </c>
+      <c r="G204" s="9" t="inlineStr">
+        <is>
+          <t>CEO round-two review</t>
+        </is>
+      </c>
+      <c r="H204" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I204" s="9" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J204" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K204" s="9" t="inlineStr">
+        <is>
+          <t>Implemented in script.js/style.css.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K201"/>
-  <dataValidations count="2">
+  <autoFilter ref="A1:K204"/>
+  <dataValidations count="4">
     <dataValidation sqref="I2:I201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Low,Normal,High,Critical"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Critical,High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16808,65 +17182,65 @@
   <dimension ref="A1:J201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="27" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Missing Info ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>What Is Missing?</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Why It Is Needed</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Who Needs To Provide It</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Deadline</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Answer / Final Info</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -19274,12 +19648,18 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J201"/>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="H2:H201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Low,Normal,High,Critical"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Critical,High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19295,71 +19675,71 @@
   <dimension ref="A1:K201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Question ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Context</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Who Should Answer</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>Answer</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Decision / Outcome</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Date Resolved</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -21967,12 +22347,18 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K201"/>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="I2:I201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Low,Normal,High,Critical"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Critical,High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21985,98 +22371,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O201"/>
+  <dimension ref="A1:O202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Schedule Update ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Day / Date</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Current Time</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>New Time</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Current Title</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>New Title</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="N1" s="8" t="inlineStr">
         <is>
           <t>Approved By</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="O1" s="8" t="inlineStr">
         <is>
           <t>Website Update Status</t>
         </is>
@@ -25482,9 +25868,86 @@
       <c r="N201" s="6" t="n"/>
       <c r="O201" s="6" t="n"/>
     </row>
+    <row r="202">
+      <c r="A202" s="9" t="inlineStr">
+        <is>
+          <t>CS-R2-001</t>
+        </is>
+      </c>
+      <c r="B202" s="9" t="inlineStr">
+        <is>
+          <t>All event days</t>
+        </is>
+      </c>
+      <c r="C202" s="9" t="inlineStr">
+        <is>
+          <t>Current schedule data</t>
+        </is>
+      </c>
+      <c r="D202" s="9" t="inlineStr">
+        <is>
+          <t>Derived daily call sheet view</t>
+        </is>
+      </c>
+      <c r="E202" s="9" t="inlineStr">
+        <is>
+          <t>Daily Call Sheet confirmation</t>
+        </is>
+      </c>
+      <c r="F202" s="9" t="inlineStr">
+        <is>
+          <t>Daily Call Sheet confirmation</t>
+        </is>
+      </c>
+      <c r="G202" s="9" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="H202" s="9" t="inlineStr">
+        <is>
+          <t>Chris Manoe</t>
+        </is>
+      </c>
+      <c r="I202" s="9" t="inlineStr">
+        <is>
+          <t>Poppy Luck / I.N.C</t>
+        </is>
+      </c>
+      <c r="J202" s="9" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="K202" s="9" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="L202" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M202" s="9" t="inlineStr">
+        <is>
+          <t>Confirm owner/support/supplier/content links for each day before final event use.</t>
+        </is>
+      </c>
+      <c r="N202" s="9" t="inlineStr">
+        <is>
+          <t>Chris Manoe</t>
+        </is>
+      </c>
+      <c r="O202" s="9" t="inlineStr">
+        <is>
+          <t>Ready for Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O201"/>
-  <dataValidations count="3">
+  <autoFilter ref="A1:O202"/>
+  <dataValidations count="6">
     <dataValidation sqref="K2:K201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
@@ -25493,6 +25956,15 @@
     </dataValidation>
     <dataValidation sqref="L2:L201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Low,Normal,High,Critical"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Critical,High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25508,83 +25980,83 @@
   <dimension ref="A1:M201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Task Update ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Task Title</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Day / Date</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Current Status</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>New Status</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>Notes / Update</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Approved By</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>Website Update Status</t>
         </is>
@@ -28592,7 +29064,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:M201"/>
-  <dataValidations count="3">
+  <dataValidations count="6">
     <dataValidation sqref="M2:M201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
@@ -28601,6 +29073,15 @@
     </dataValidation>
     <dataValidation sqref="J2:J201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -28616,95 +29097,95 @@
   <dimension ref="A1:O203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Contact Update ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Correct Name</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Company / Team</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>On-Site or Remote</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>Main Responsibility</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="N1" s="8" t="inlineStr">
         <is>
           <t>Approved By</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="O1" s="8" t="inlineStr">
         <is>
           <t>Website Update Status</t>
         </is>
@@ -32110,24 +32591,47 @@
       <c r="N201" s="6" t="n"/>
       <c r="O201" s="6" t="n"/>
     </row>
+    <row r="202">
+      <c r="A202" s="9" t="n"/>
+      <c r="B202" s="9" t="n"/>
+      <c r="C202" s="9" t="n"/>
+      <c r="D202" s="9" t="n"/>
+      <c r="E202" s="9" t="n"/>
+      <c r="F202" s="9" t="n"/>
+      <c r="G202" s="9" t="n"/>
+      <c r="H202" s="9" t="n"/>
+      <c r="I202" s="9" t="n"/>
+      <c r="J202" s="9" t="n"/>
+      <c r="K202" s="9" t="n"/>
+      <c r="L202" s="9" t="n"/>
+      <c r="M202" s="9" t="n"/>
+      <c r="N202" s="9" t="n"/>
+      <c r="O202" s="9" t="n"/>
+    </row>
     <row r="203">
-      <c r="A203" s="7" t="inlineStr">
+      <c r="A203" s="12" t="inlineStr">
         <is>
           <t>Chris Manoe rule: there is only one Chris. Do not add Chris Minot, CM, or Chris M.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O201"/>
+  <autoFilter ref="A1:O203"/>
   <mergeCells count="1">
     <mergeCell ref="A203:O203"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="M2:M201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -32143,113 +32647,113 @@
   <dimension ref="A1:R201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="34" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="34" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="25" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="23" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Supplier Update ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Supplier Name</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Supplier Type</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Contact Person</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Internal Owner</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Day / Date</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Arrival Time</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Setup Time</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>Active Time</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="11" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="11" t="inlineStr">
         <is>
           <t>Responsibility</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="N1" s="11" t="inlineStr">
         <is>
           <t>Open Item / Question</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="O1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="P1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="Q1" s="8" t="inlineStr">
         <is>
           <t>Approved By</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="R1" s="8" t="inlineStr">
         <is>
           <t>Website Update Status</t>
         </is>
@@ -36257,12 +36761,18 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:R201"/>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="O2:O201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
     <dataValidation sqref="R2:R201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R2:R5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -36278,83 +36788,83 @@
   <dimension ref="A1:M201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Podcast Update ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Day / Date</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Guest</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Host</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Crew</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Production Needs</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Current Status</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>New Status</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Approved By</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>Website Update Status</t>
         </is>
@@ -39362,7 +39872,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:M201"/>
-  <dataValidations count="3">
+  <dataValidations count="6">
     <dataValidation sqref="M2:M201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
@@ -39372,6 +39882,15 @@
     <dataValidation sqref="J2:J201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Needs Confirmation,Approved,Ready for Codex,Added to Website,Rejected / Do Not Add,Waiting on Info,Complete"</formula1>
     </dataValidation>
+    <dataValidation sqref="I2:I5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Missing,Needs Confirmation,Waiting on Person,Answered,Approved,Added to Website,Not Needed"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync HORIZONS final schedule and materials updates
</commit_message>
<xml_diff>
--- a/HORIZONS_Website_Update_Tracker.xlsx
+++ b/HORIZONS_Website_Update_Tracker.xlsx
@@ -539,7 +539,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -547,7 +546,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -4015,7 +4013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K201"/>
+  <dimension ref="A1:K203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6687,6 +6685,120 @@
       <c r="I201" s="6" t="n"/>
       <c r="J201" s="6" t="n"/>
       <c r="K201" s="6" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>DOC-SYNC-001</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>HORIZONS Website Final Schedule Sync Workbook</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Source Data</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Latest workbook source for website sync</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>horizons-website-final-schedule-sync-for-codex.xlsx</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>assets/documents/horizons-website-final-schedule-sync-for-codex.xlsx</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Samuel Price</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Documents / Source Data</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>Copied into assets/documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>DOC-SYNC-002</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>HORIZONS Swag Delivery Brief</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Swag / Guest Materials</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Reference for room drops, swag, and guest materials</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>horizons-swag-delivery-brief.pdf</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>assets/documents/horizons-swag-delivery-brief.pdf</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>BE GOOD / HORIZONS team</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>Documents / Swag / Guest Materials</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>Copied into assets/documents</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K201"/>
@@ -14309,7 +14421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K204"/>
+  <dimension ref="A1:K207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17150,6 +17262,177 @@
       <c r="K204" s="9" t="inlineStr">
         <is>
           <t>Implemented in script.js/style.css.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>WCR-SYNC-001</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>29 May 2026</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Schedule / Call Sheet</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Latest workbook not fully reflected</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Sync latest 310-row schedule, add Saturday 6 June, and use AM/PM display</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Latest final schedule sync workbook</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Applied to content.json; unresolved source gaps remain Needs Confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>WCR-SYNC-002</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>29 May 2026</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Guest Materials &amp; Experience</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Swag section too narrow</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Expand to Guest Materials &amp; Experience and add tote bags, crew shirts, easel boards, signage, menus</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Latest user revision and assets</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Assets linked; missing files remain placeholders</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>WCR-SYNC-003</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>29 May 2026</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Call Sheet</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Weather needed</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Add weather module placeholder for Six Senses Ibiza / Ibiza</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Latest user revision</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>Live weather API/source still needed</t>
         </is>
       </c>
     </row>
@@ -32644,7 +32927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R201"/>
+  <dimension ref="A1:R203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -36759,6 +37042,154 @@
       <c r="Q201" s="6" t="n"/>
       <c r="R201" s="6" t="n"/>
     </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>SUP-SYNC-001</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Mobile Casino / Poker</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Supplier / Performer</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Contact needed</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr"/>
+      <c r="F202" t="inlineStr"/>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Dawn Ramsden / BE GOOD</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Wednesday 10 June</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr"/>
+      <c r="J202" t="inlineStr"/>
+      <c r="K202" t="inlineStr"/>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>Arcade</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>Poker/casino setup</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>Confirm setup 15:00-16:00 vs later delivery and 33 chairs</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>Added from final revision</t>
+        </is>
+      </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>Samuel / Dawn</t>
+        </is>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>SUP-SYNC-002</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>BE GOOD</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Operations / Logistics</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Ben Eddon-Carruthers / Cheryl Leno</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>See Contacts tab</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr"/>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Samuel Price</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>All event</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr"/>
+      <c r="J203" t="inlineStr"/>
+      <c r="K203" t="inlineStr"/>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>Six Senses Ibiza / HORIZONS House</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>Room drops, logistics, guest materials</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>Confirm all day/time details and final file uploads</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t>Company spelling standardized as BE GOOD</t>
+        </is>
+      </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>Samuel</t>
+        </is>
+      </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R201"/>
   <dataValidations count="4">

</xml_diff>

<commit_message>
Add HORIZONS operations sections and Slack integration stub
</commit_message>
<xml_diff>
--- a/HORIZONS_Website_Update_Tracker.xlsx
+++ b/HORIZONS_Website_Update_Tracker.xlsx
@@ -4013,7 +4013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K203"/>
+  <dimension ref="A1:K204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6797,6 +6797,59 @@
       <c r="K203" t="inlineStr">
         <is>
           <t>Copied into assets/documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>DOC-MISSING-FILES-001</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Missing Files Tracker</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Source Data</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Expanded missing files tracker for call sheets, Cvent, speaker content, signage, staff, entertainment, playlists, podcast, and venue files</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>content.json missingFiles</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr"/>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Samuel Price</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Missing Files section</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Keep approved files in Documents section</t>
         </is>
       </c>
     </row>
@@ -14421,7 +14474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K207"/>
+  <dimension ref="A1:K210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17433,6 +17486,177 @@
       <c r="K207" t="inlineStr">
         <is>
           <t>Live weather API/source still needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>REQ-SLACK-001</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>29 May 2026</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Slack Integration</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Add Slack-safe source-of-truth communication layer with channel map and copy update actions</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Add Slack section, channel mapping, and no-secret webhook guidance</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Leadership feedback</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Webhook URLs must be configured server-side only</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>REQ-LOC-001</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>29 May 2026</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Location Schedules</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Need location-specific and restaurant-specific views</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Add Location Schedules and Restaurant Schedules sections from master schedule data</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Leadership feedback</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Uses content.json locationSchedules and restaurantSchedules</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>REQ-CONTENT-001</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>29 May 2026</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Speakers / Cvent / Entertainment</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Need speaker content, Cvent audit, entertainment, playlists, rehearsals and signage models</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Add compact operational sections and data records</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Leadership feedback</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>Unconfirmed data stays Needs Confirmation/File Needed</t>
         </is>
       </c>
     </row>
@@ -29377,7 +29601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O203"/>
+  <dimension ref="A1:O204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -32895,6 +33119,71 @@
       <c r="A203" s="12" t="inlineStr">
         <is>
           <t>Chris Manoe rule: there is only one Chris. Do not add Chris Minot, CM, or Chris M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>CONTACT-SAMUEL-ROLE-001</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Samuel Price</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Samuel Price</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Podcast Lead / Executive Assistant to Chris Manoe / Website Development &amp; Software Lead / Infrastructure &amp; Systems Support Lead</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>HORIZONS</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Leadership / Production / Systems</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr"/>
+      <c r="H204" t="inlineStr"/>
+      <c r="I204" t="inlineStr"/>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>On-site / support</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Podcast, Chris support, website/software, infrastructure/systems</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>Updated from latest leadership brief</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>Added to Website</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>Added to contact card and staff list</t>
         </is>
       </c>
     </row>
@@ -37063,8 +37352,6 @@
           <t>Contact needed</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr"/>
-      <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
           <t>Dawn Ramsden / BE GOOD</t>
@@ -37075,9 +37362,6 @@
           <t>Wednesday 10 June</t>
         </is>
       </c>
-      <c r="I202" t="inlineStr"/>
-      <c r="J202" t="inlineStr"/>
-      <c r="K202" t="inlineStr"/>
       <c r="L202" t="inlineStr">
         <is>
           <t>Arcade</t>
@@ -37140,7 +37424,6 @@
           <t>See Contacts tab</t>
         </is>
       </c>
-      <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
           <t>Samuel Price</t>
@@ -37151,9 +37434,6 @@
           <t>All event</t>
         </is>
       </c>
-      <c r="I203" t="inlineStr"/>
-      <c r="J203" t="inlineStr"/>
-      <c r="K203" t="inlineStr"/>
       <c r="L203" t="inlineStr">
         <is>
           <t>Six Senses Ibiza / HORIZONS House</t>

</xml_diff>

<commit_message>
Refine HORIZONS onsite UX, navigation, comments, and programme sections
</commit_message>
<xml_diff>
--- a/HORIZONS_Website_Update_Tracker.xlsx
+++ b/HORIZONS_Website_Update_Tracker.xlsx
@@ -6831,7 +6831,6 @@
           <t>content.json missingFiles</t>
         </is>
       </c>
-      <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr">
         <is>
           <t>Samuel Price</t>
@@ -14548,95 +14547,403 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n"/>
-      <c r="B2" s="5" t="n"/>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="5" t="n"/>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>UX-ONSITE-001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Hero / Header</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Visible hero repeated HORIZONS Ibiza 2026 beneath the official logo.</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Remove repeated visible event title and centre hero content around the official logo.</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Chris/Samuel onsite review: reduce duplication and keep the brand moment calmer.</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Implemented in index.html/style.css; official event name remains in source metadata.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
-      <c r="J3" s="6" t="n"/>
-      <c r="K3" s="6" t="n"/>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>UX-ONSITE-002</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Leadership and admin sections were mixed together in a long navigation list.</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Reorder navigation into Start, Operations, People, Programme, Guest Experience, and Admin groups.</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Make mobile navigation easier for executives and onsite operators.</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Decisions moved higher; admin/developer tools moved lower.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>UX-ONSITE-003</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Comments / Updates</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Updates could be added but resolution/archiving needed clearer actions.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Add Mark Resolved, Archive, Reopen, Slack channel selector, and urgent preview to update threads.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Team needs to clear handled items without deleting history.</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Shared backend remains source for updates; archive/history stays visible.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="n"/>
-      <c r="K5" s="6" t="n"/>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>UX-ONSITE-004</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Call Sheet</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Weather and emergency cards stacked on desktop and top notes pushed the timeline down.</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Use side-by-side weather/emergency cards on desktop, compact notes, day/date tabs, and current time marker.</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Improve onsite call sheet scanning.</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Weather cache key refreshed after coordinate/location correction.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>UX-ONSITE-005</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Programme Sections</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Podcast, speakers, entertainment, playlists, location schedules, and restaurants needed clearer grouping.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Group podcast by day/episode; speakers by location/day; locations/restaurants by day; separate live entertainment from curated playlists.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Reduce scrolling and avoid mixing background music with live performers.</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Detailed unknown podcast/speaker fields remain Needs Confirmation.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="n"/>
-      <c r="K7" s="6" t="n"/>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>UX-ONSITE-006</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Admin Tools</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Admin-heavy sections were prominent in the main flow.</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Move Cvent, Missing Files, Slack, Data Health, Duplicate Review, and Site Audit into the lower admin navigation group.</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Keep the main team experience calmer.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Admin records remain available.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>UX-ONSITE-007</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>HORIZONS Studio</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Standalone HORIZONS Studio operational section was not useful.</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Hide/remove standalone HORIZONS Studio section while retaining Studio as location/source/programme data.</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Latest review requested removal of standalone section only.</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>HORIZONS Studio still appears in location schedules, speakers, rehearsals, call sheet, and data records.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
@@ -17754,136 +18061,488 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n"/>
-      <c r="B2" s="5" t="n"/>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="5" t="n"/>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>MI-ONSITE-001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Contacts / Travel</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Confirm Eve Dusek name, role, and contact details.</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Approved display name is Eve Dusek; role currently tracked as COO of Aream &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Samuel / Aream &amp; Co.</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr"/>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr"/>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Do not use the old name in live display unless confirmed as a separate person.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
-      <c r="J3" s="6" t="n"/>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>MI-ONSITE-002</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Who Do I Call / Emergency</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Health &amp; Safety owner and emergency escalation process.</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Who Do I Call needs explicit Health &amp; Safety coverage.</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Samuel / Chris / Venue</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr"/>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Include phone, WhatsApp, venue contact, and escalation notes.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>MI-ONSITE-003</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Locations / Maps</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Venue map, exact internal pins, room layouts, seating plans, and Google Maps links.</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Location cards and call sheet need exact maps without guessing.</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Venue / Operations</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr"/>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Use Google Maps Link Needed / Exact pin needed until supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="n"/>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>MI-ONSITE-004</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Confirm final weather coordinate / event hotel pin.</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Open-Meteo is using Six Senses Ibiza / Xarraca Bay coordinates as a temporary confirmed-nearby point.</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Samuel / Venue</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Weather location needs confirmation remains in notes.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>MI-ONSITE-005</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>HORIZONS House</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Display cabinet image.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Reception Display section needs the glass display cabinet image.</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Creative / Guest Experience</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>File Needed</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Placeholder remains on site.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="n"/>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>MI-ONSITE-006</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Room Drops</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Confirm Pulsio / Poltio product name and room-drop placement.</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Review notes mention Poltio; source image appears massage-gun/Pulsio-like.</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Samuel / Guest Experience</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Do not finalize naming until confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>MI-ONSITE-007</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Guest Materials</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Crew shirts data/image confirmation.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Current crew shirt item may be incorrect.</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Samuel / Guest Experience</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Flagged on site.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
-      <c r="J9" s="6" t="n"/>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>MI-ONSITE-008</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Speakers / Podcast</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Final speaker content and podcast guest/company/prep ownership.</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Speaker grouping and podcast episode cards need final content.</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Samuel / Production</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>Includes guest runner, prep owner, microphone and powder/makeup checks.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>MI-ONSITE-009</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Rehearsals</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>HORIZONS Studio rehearsal timing for 8 June.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Placeholder added with Time needed.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Confirm required people and owner.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="n"/>
-      <c r="I11" s="6" t="n"/>
-      <c r="J11" s="6" t="n"/>
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>MI-ONSITE-010</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Signage / Wayfinding</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Wayfinding artwork, A1 boards, three totem locations, two wall foam board locations, and placement map.</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Clownfish need exact install placement.</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Creative / Clownfish</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>File Needed</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>Site has placeholders for Map Needed / Location Needed / Placement Needed.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>MI-ONSITE-011</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Staff / Cvent / Slack</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Staff corrections, Cvent export, and Slack production routing approval.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Admin/developer setup is ready but should not be activated broadly without approval.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Samuel / Chris</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Production Slack routes remain disabled/test-mode until approved.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
@@ -20253,43 +20912,127 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n"/>
-      <c r="B2" s="5" t="n"/>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="5" t="n"/>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Q-ONSITE-001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Weather / Location</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Is the Open-Meteo coordinate the exact event hotel pin or only a nearby Six Senses Ibiza reference?</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Current site uses Six Senses Ibiza / Xarraca Bay coordinates and labels final pin as needing confirmation.</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Samuel / Venue</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr"/>
+      <c r="G2" s="5" t="inlineStr"/>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr"/>
+      <c r="K2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
-      <c r="J3" s="6" t="n"/>
-      <c r="K3" s="6" t="n"/>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Q-ONSITE-002</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Slack</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>When should production Slack routes be activated beyond #horizons-test?</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Website supports channel selection but production webhooks should not be enabled without approval.</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Samuel / Chris</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Q-ONSITE-003</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Room Drops</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Should the product be displayed as Pulsio, Poltio, or another approved name?</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Latest notes used Poltio; asset resembles massage-gun/Pulsio item.</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Guest Experience</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Needs Confirmation</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr"/>
+      <c r="K4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n"/>
@@ -33153,9 +33896,6 @@
           <t>Leadership / Production / Systems</t>
         </is>
       </c>
-      <c r="G204" t="inlineStr"/>
-      <c r="H204" t="inlineStr"/>
-      <c r="I204" t="inlineStr"/>
       <c r="J204" t="inlineStr">
         <is>
           <t>On-site / support</t>

</xml_diff>